<commit_message>
Updated HRV_grids_kan10 model - 2026-08-26 15:56
</commit_message>
<xml_diff>
--- a/VerveStacks_HRV_grids_kan10/Sets-vervestacks.xlsx
+++ b/VerveStacks_HRV_grids_kan10/Sets-vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_HRV_grids_kan10\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1DF2BDEE-71F2-4E34-B2D6-58160B578B6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{ABA857A8-24D0-44F2-BB11-86B77DD485F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1467,7 +1467,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C78A754-EB1B-4CE4-A246-CC8E81627ED9}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35DD0B8B-0DDB-4E44-A6C9-5E89E9F87939}">
   <dimension ref="B9:E53"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>

</xml_diff>